<commit_message>
freeze published workbook state
</commit_message>
<xml_diff>
--- a/data/pipeline-command-center.xlsx
+++ b/data/pipeline-command-center.xlsx
@@ -2500,7 +2500,11 @@
       <c r="H3" t="n">
         <v>55000</v>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2517,14 +2521,18 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr">
         <is>
           <t>Opportunities-2026: Hot_Leads</t>
@@ -2541,7 +2549,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -2576,7 +2584,11 @@
       </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Commercial Manager</t>
+        </is>
+      </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr"/>
@@ -2661,28 +2673,32 @@
           <t>2025-02-05</t>
         </is>
       </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>00/01/1900</t>
-        </is>
-      </c>
+      <c r="BJ3" t="inlineStr"/>
       <c r="BK3" t="inlineStr">
         <is>
-          <t>2023-01-01</t>
-        </is>
-      </c>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>2023-01-08</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>Commercial Manager</t>
+        </is>
+      </c>
       <c r="BO3" t="inlineStr"/>
       <c r="BP3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ3" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="BQ3" t="inlineStr"/>
       <c r="BR3" t="inlineStr">
         <is>
           <t>Evolution: 15% + Premium: 1% - 5% Ezugi: 13% + Premium: 1% - 3% Slots: 12% Premium: 15%</t>
@@ -2693,23 +2709,11 @@
           <t>Client Legal</t>
         </is>
       </c>
-      <c r="BT3" t="inlineStr">
-        <is>
-          <t>www</t>
-        </is>
-      </c>
-      <c r="BU3" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
       <c r="BV3" t="inlineStr"/>
       <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="BX3" t="inlineStr"/>
       <c r="CR3" t="inlineStr"/>
       <c r="CT3" t="inlineStr"/>
       <c r="CU3" t="n">
@@ -55247,7 +55251,11 @@
         <v>1</v>
       </c>
       <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Send Proposal</t>
+        </is>
+      </c>
       <c r="P180" t="inlineStr">
         <is>
           <t>Opportunities-2026: Accounts</t>
@@ -55328,10 +55336,18 @@
       <c r="AJ180" t="inlineStr"/>
       <c r="AK180" t="inlineStr"/>
       <c r="AL180" t="inlineStr"/>
-      <c r="AM180" t="inlineStr"/>
+      <c r="AM180" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
       <c r="AN180" t="inlineStr"/>
       <c r="AO180" t="inlineStr"/>
-      <c r="AP180" t="inlineStr"/>
+      <c r="AP180" t="inlineStr">
+        <is>
+          <t>Creedz</t>
+        </is>
+      </c>
       <c r="AQ180" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -69701,7 +69717,11 @@
       <c r="H234" t="n">
         <v>25000</v>
       </c>
-      <c r="I234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="J234" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -69725,7 +69745,11 @@
           <t>Prospect</t>
         </is>
       </c>
-      <c r="O234" t="inlineStr"/>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>contact client</t>
+        </is>
+      </c>
       <c r="P234" t="inlineStr">
         <is>
           <t>Opportunities-2026: Hot_Leads</t>
@@ -69772,9 +69796,17 @@
           <t>1xbet</t>
         </is>
       </c>
-      <c r="AC234" t="inlineStr"/>
+      <c r="AC234" t="inlineStr">
+        <is>
+          <t>1Xbet</t>
+        </is>
+      </c>
       <c r="AD234" t="inlineStr"/>
-      <c r="AE234" t="inlineStr"/>
+      <c r="AE234" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
       <c r="AF234" t="inlineStr"/>
       <c r="AG234" t="inlineStr"/>
       <c r="AH234" t="inlineStr"/>
@@ -69848,13 +69880,29 @@
       <c r="BH234" t="inlineStr"/>
       <c r="BI234" t="inlineStr"/>
       <c r="BJ234" t="inlineStr"/>
-      <c r="BK234" t="inlineStr"/>
-      <c r="BL234" t="inlineStr"/>
-      <c r="BM234" t="inlineStr"/>
-      <c r="BN234" t="inlineStr"/>
+      <c r="BK234" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="BL234" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="BM234" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="BN234" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
       <c r="BO234" t="inlineStr"/>
       <c r="BP234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ234" t="inlineStr"/>
       <c r="BR234" t="inlineStr"/>
@@ -69865,7 +69913,7 @@
       </c>
       <c r="BT234" t="inlineStr">
         <is>
-          <t>1xbet.com</t>
+          <t>https://1xbet.com</t>
         </is>
       </c>
       <c r="BU234" t="inlineStr"/>
@@ -70473,7 +70521,11 @@
       <c r="H237" t="n">
         <v>25000</v>
       </c>
-      <c r="I237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="J237" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -70497,7 +70549,11 @@
           <t>Prospect</t>
         </is>
       </c>
-      <c r="O237" t="inlineStr"/>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>Contact Client</t>
+        </is>
+      </c>
       <c r="P237" t="inlineStr">
         <is>
           <t>Opportunities-2026: Hot_Leads</t>
@@ -70545,8 +70601,16 @@
         </is>
       </c>
       <c r="AC237" t="inlineStr"/>
-      <c r="AD237" t="inlineStr"/>
-      <c r="AE237" t="inlineStr"/>
+      <c r="AD237" t="inlineStr">
+        <is>
+          <t>Bing Par</t>
+        </is>
+      </c>
+      <c r="AE237" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
       <c r="AF237" t="inlineStr"/>
       <c r="AG237" t="inlineStr"/>
       <c r="AH237" t="inlineStr"/>
@@ -70621,12 +70685,24 @@
       <c r="BI237" t="inlineStr"/>
       <c r="BJ237" t="inlineStr"/>
       <c r="BK237" t="inlineStr"/>
-      <c r="BL237" t="inlineStr"/>
-      <c r="BM237" t="inlineStr"/>
-      <c r="BN237" t="inlineStr"/>
+      <c r="BL237" t="inlineStr">
+        <is>
+          <t>Biweekly</t>
+        </is>
+      </c>
+      <c r="BM237" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="BN237" t="inlineStr">
+        <is>
+          <t>Erick</t>
+        </is>
+      </c>
       <c r="BO237" t="inlineStr"/>
       <c r="BP237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ237" t="inlineStr"/>
       <c r="BR237" t="inlineStr"/>
@@ -70637,7 +70713,7 @@
       </c>
       <c r="BT237" t="inlineStr">
         <is>
-          <t>bingopar.com.py</t>
+          <t>https:bingopar.py</t>
         </is>
       </c>
       <c r="BU237" t="inlineStr"/>

</xml_diff>

<commit_message>
sync workbook data and tighten integrity checks
</commit_message>
<xml_diff>
--- a/data/pipeline-command-center.xlsx
+++ b/data/pipeline-command-center.xlsx
@@ -10645,7 +10645,11 @@
         </is>
       </c>
       <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Erick Mendez</t>
+        </is>
+      </c>
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="inlineStr"/>
@@ -10742,12 +10746,12 @@
       </c>
       <c r="BL26" t="inlineStr">
         <is>
-          <t>Weekly</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="BM26" t="inlineStr">
         <is>
-          <t>2023-01-08</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="BN26" t="inlineStr">
@@ -54159,7 +54163,11 @@
           <t>Impresora Internacional de Valores SAIC (IVISA)</t>
         </is>
       </c>
-      <c r="O172" t="inlineStr"/>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>contact Shai</t>
+        </is>
+      </c>
       <c r="P172" t="inlineStr">
         <is>
           <t>Opportunities-2026: Accounts</t>
@@ -54308,7 +54316,7 @@
       <c r="BJ172" t="inlineStr"/>
       <c r="BK172" t="inlineStr">
         <is>
-          <t>2025-04-15</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="BL172" t="inlineStr">
@@ -54328,7 +54336,7 @@
       </c>
       <c r="BO172" t="inlineStr"/>
       <c r="BP172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ172" t="inlineStr"/>
       <c r="BR172" t="inlineStr">
@@ -54481,7 +54489,11 @@
           <t>Paradise Games Bahamas Ltd</t>
         </is>
       </c>
-      <c r="O173" t="inlineStr"/>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>provide content certificates</t>
+        </is>
+      </c>
       <c r="P173" t="inlineStr">
         <is>
           <t>Opportunities-2026: Accounts</t>
@@ -54513,7 +54525,7 @@
         <v>1</v>
       </c>
       <c r="X173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y173" t="n">
         <v>0</v>
@@ -54657,7 +54669,11 @@
       <c r="BW173" t="inlineStr"/>
       <c r="BX173" t="inlineStr"/>
       <c r="CR173" t="inlineStr"/>
-      <c r="CT173" t="inlineStr"/>
+      <c r="CT173" t="inlineStr">
+        <is>
+          <t>Paradise Games Bahamas Ltd</t>
+        </is>
+      </c>
       <c r="CU173" t="n">
         <v>30</v>
       </c>
@@ -59439,7 +59455,11 @@
       <c r="H191" t="n">
         <v>25000</v>
       </c>
-      <c r="I191" t="inlineStr"/>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
       <c r="J191" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -59514,7 +59534,11 @@
           <t>Mas1x2.com</t>
         </is>
       </c>
-      <c r="AC191" t="inlineStr"/>
+      <c r="AC191" t="inlineStr">
+        <is>
+          <t>Mas1x2.com</t>
+        </is>
+      </c>
       <c r="AD191" t="inlineStr"/>
       <c r="AE191" t="inlineStr"/>
       <c r="AF191" t="inlineStr"/>
@@ -59604,15 +59628,27 @@
       <c r="BJ191" t="inlineStr"/>
       <c r="BK191" t="inlineStr">
         <is>
-          <t>2025-06-18</t>
-        </is>
-      </c>
-      <c r="BL191" t="inlineStr"/>
-      <c r="BM191" t="inlineStr"/>
-      <c r="BN191" t="inlineStr"/>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="BL191" t="inlineStr">
+        <is>
+          <t>Biweekly</t>
+        </is>
+      </c>
+      <c r="BM191" t="inlineStr">
+        <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="BN191" t="inlineStr">
+        <is>
+          <t>LATAM Workspace Admin</t>
+        </is>
+      </c>
       <c r="BO191" t="inlineStr"/>
       <c r="BP191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ191" t="inlineStr"/>
       <c r="BR191" t="inlineStr"/>
@@ -59623,7 +59659,11 @@
       <c r="BW191" t="inlineStr"/>
       <c r="BX191" t="inlineStr"/>
       <c r="CR191" t="inlineStr"/>
-      <c r="CT191" t="inlineStr"/>
+      <c r="CT191" t="inlineStr">
+        <is>
+          <t>Mas1x2.com</t>
+        </is>
+      </c>
       <c r="CU191" t="n">
         <v>30</v>
       </c>
@@ -81129,7 +81169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81242,17 +81282,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>task-1777957030755-e79e1e</t>
+          <t>task-1777957030757-fb10ae</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TSK-2023-0005</t>
+          <t>TSK-2023-0006</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Weekly follow-up 1 · Caribevivo</t>
+          <t>Weekly follow-up 2 · Caribevivo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -81272,7 +81312,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023-01-08</t>
+          <t>+252026-05</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -81325,23 +81365,31 @@
           <t>Cold Not started Not started Not started</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2026-05-05T13:29:22.374Z</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-05-05T13:29:22.374Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>task-1777957030757-fb10ae</t>
+          <t>task-1777957030757-a93113</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TSK-2023-0006</t>
+          <t>TSK-2023-0007</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Weekly follow-up 2 · Caribevivo</t>
+          <t>Weekly follow-up 3 · Caribevivo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -81361,7 +81409,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2023-01-15</t>
+          <t>2023-01-22</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -81420,17 +81468,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>task-1777957030757-a93113</t>
+          <t>task-1777957030757-801e9f</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TSK-2023-0007</t>
+          <t>TSK-2023-0008</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Weekly follow-up 3 · Caribevivo</t>
+          <t>Weekly follow-up 4 · Caribevivo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -81450,7 +81498,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023-01-22</t>
+          <t>2023-01-29</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -81509,17 +81557,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>task-1777957030757-801e9f</t>
+          <t>task-1777989208027-4c9923</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TSK-2023-0008</t>
+          <t>TSK-2025-0009</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Weekly follow-up 4 · Caribevivo</t>
+          <t>Biweekly follow-up 1 · Mas1x2.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -81539,7 +81587,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2023-01-29</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -81549,28 +81597,28 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>deal-1777531025.680739</t>
+          <t>deal-1777531025.684233</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Caribevivo</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Caribevivo</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Caribevivo</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="O5" t="n">
@@ -81579,17 +81627,17 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-05 Weekly follow-up plan scheduled</t>
+          <t>2026-05-05 Biweekly follow-up plan scheduled</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Complete handover date set and live owner assigned before moving this account to Performance Review.</t>
+          <t>Send proposal</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Cold Not started Not started Not started</t>
+          <t>Negotiation Not started Not started Not started Send proposal</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -81598,17 +81646,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>task-1777941298665-a72128</t>
+          <t>task-1777989208031-63e1ea</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TSK-2026-0002</t>
+          <t>TSK-2025-0010</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Monthly follow-up 1 · Stake</t>
+          <t>Biweekly follow-up 2 · Mas1x2.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -81628,7 +81676,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2025-07-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -81638,28 +81686,28 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>deal-1777531025.687534</t>
+          <t>deal-1777531025.684233</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="O6" t="n">
@@ -81668,32 +81716,36 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+          <t>2026-05-05 Biweekly follow-up plan scheduled</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
+          <t>Send proposal</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Negotiation Not started Not started Not started Send proposal</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>task-1777941298666-c016c7</t>
+          <t>task-1777989208032-da3900</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TSK-2026-0003</t>
+          <t>TSK-2025-0011</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Monthly follow-up 2 · Stake</t>
+          <t>Biweekly follow-up 3 · Mas1x2.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -81713,7 +81765,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2025-07-30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -81723,28 +81775,28 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>deal-1777531025.687534</t>
+          <t>deal-1777531025.684233</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="O7" t="n">
@@ -81753,32 +81805,36 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+          <t>2026-05-05 Biweekly follow-up plan scheduled</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+          <t>Send proposal</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Negotiation Not started Not started Not started Send proposal</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>task-1777941298666-6b445d</t>
+          <t>task-1777989208034-702c75</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TSK-2026-0004</t>
+          <t>TSK-2025-0012</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Monthly follow-up 3 · Stake</t>
+          <t>Biweekly follow-up 4 · Mas1x2.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -81798,7 +81854,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2025-08-13</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -81808,28 +81864,28 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>deal-1777531025.687534</t>
+          <t>deal-1777531025.684233</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>Mas1x2.com</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="O8" t="n">
@@ -81838,17 +81894,369 @@
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+          <t>2026-05-05 Biweekly follow-up plan scheduled</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>Send proposal</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Negotiation Not started Not started Not started Send proposal</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>task-1777941298665-a72128</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TSK-2026-0002</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Monthly follow-up 1 · Stake</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>LATAM Workspace Admin</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>deal-1777531025.687534</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>task-1777941298666-c016c7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TSK-2026-0003</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Monthly follow-up 2 · Stake</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>LATAM Workspace Admin</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>deal-1777531025.687534</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>task-1777941298666-6b445d</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TSK-2026-0004</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Monthly follow-up 3 · Stake</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>LATAM Workspace Admin</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>deal-1777531025.687534</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-05-05 Monthly follow-up plan scheduled</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Complete account context documented and future opportunities logged before moving this account to Performance Review.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>task-1777957030755-e79e1e</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TSK-2023-0005</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Weekly follow-up 1 · Caribevivo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2023-01-08</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>LATAM Workspace Admin</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>deal-1777531025.680739</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Caribevivo</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Caribevivo</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Caribevivo</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-05-05 Weekly follow-up plan scheduled</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Complete handover date set and live owner assigned before moving this account to Performance Review.</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Cold Not started Not started Not started</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2026-05-05T13:23:33.452Z</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -82129,7 +82537,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>